<commit_message>
Import verified commercial delivery and reservation links from June audit.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
+++ b/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
@@ -1905,6 +1905,11 @@
           <t>https://oshione.de/ ; https://www.berlin-glutenfrei.de/glutenfrei-berlin-restaurants/oshione</t>
         </is>
       </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="BB9" t="n">
         <v>52.486077</v>
       </c>
@@ -2635,6 +2640,11 @@
       <c r="AJ14" t="b">
         <v>0</v>
       </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>https://www.thefork.de/restaurant/trattoria-senza-gluten-free-restaurant-r837761</t>
+        </is>
+      </c>
       <c r="AO14" t="inlineStr">
         <is>
           <t>Specialist directory</t>
@@ -2648,6 +2658,11 @@
       <c r="AQ14" t="inlineStr">
         <is>
           <t>https://www.berlin-glutenfrei.de/glutenfrei-berlin-restaurants/trattoria-senza ; https://www.eatthisdot.com/restaurant/trattoria-senza</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="BB14" t="n">
@@ -10320,7 +10335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10362,6 +10377,86 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DL-DE-TOP4-003-WOLT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DE-TOP4-003</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Oshione</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Wolt</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://wolt.com/de/deu/berlin/venue/oshione-glutenfree-a50db1</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Wolt venue/product page indexed; page states Oshione Glutenfree, Katzbachstraße 25, 100% glutenfrei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DL-DE-TOP4-008-WOLT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DE-TOP4-008</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trattoria Senza</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Wolt</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://wolt.com/de/deu/berlin/restaurant/trattoria-senza-hannoversche-str-berlin</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Wolt page indexed for Trattoria Senza, Hannoversche Str., Berlin.</t>
         </is>
       </c>
     </row>
@@ -10376,7 +10471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10418,6 +10513,46 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RS-DE-TOP4-008-THEFORK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DE-TOP4-008</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Trattoria Senza</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TheFork</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.thefork.de/restaurant/trattoria-senza-gluten-free-restaurant-r837761</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TheFork page indexed for Trattoria Senza - Gluten Free Restaurant, Hannoversche Str. 1 Berlin.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Import official website descriptions from ES/DE audit.
Add apply-descriptions pipeline and rebuild bundled data so all 190 venues have German copy.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
+++ b/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
@@ -828,7 +828,7 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Official source states the bakery bakes exclusively gluten-free; Frankfurt location and address are listed on official site.</t>
+          <t>Café / Pâtisserie / Bakery in Frankfurt am Main. Official source states the bakery bakes exclusively gluten-free; Frankfurt location and address are listed on official site.</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Official site positions the restaurant with gluten-free branding and address; specialist/current community sources describe it as 100% gluten-free. Direct written confirmation still recommended for app maximum assurance.</t>
+          <t>Restaurant / Vietnamese in Frankfurt am Main. Official site positions the restaurant with gluten-free branding and address; specialist/current community sources describe it as 100% gluten-free. Direct written confirmation still recommended for app maximum assurance.</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Official site lists current address; Zöliakie Austausch states everything is 100% gluten-free. Old sources list Lindley/Oederweg, so location list must be rechecked before import.</t>
+          <t>Café / Bakery / Raw cakes in Frankfurt am Main. Official site lists current address; Zöliakie Austausch states everything is 100% gluten-free. Old sources list Lindley/Oederweg, so location list must be rechecked before import.</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Current operator states she took over Kaffeebar by Alex and offers gluten-free specialties; legacy sources describe the location as completely gluten-free. Current official wording says gluten-free specialties/options, so direct confirmation recommended before hard 100%-GF badge.</t>
+          <t>Café / Bakery / Brunch in Frankfurt am Main. Current operator states she took over Kaffeebar by Alex and offers gluten-free specialties; legacy sources describe the location as completely gluten-free. Current official wording says gluten-free specialties/options, so direct confirmation recommended before hard 100%-GF badge.</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Accepted for import as Frankfurt Rhein-Main / Bad Homburg. Official site describes a gluten-free café/products; specialist source says all products are gluten-free. City is Bad Homburg, not Frankfurt am Main, so region/city filters must show it as Bad Homburg.</t>
+          <t>Café / Superfood / Bowls in Bad Homburg vor der Höhe. Accepted for import as Frankfurt Rhein-Main / Bad Homburg. Official site describes a gluten-free café/products; specialist source says all products are gluten-free. City is Bad Homburg, not Frankfurt am Main, so region/city filters must show it as Bad Homburg.</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists AERA Charlottenburg as vollständig glutenfreies Angebot and states that the bakery bakes exclusively gluten-free; AERA official site markets 100% gluten-free sourdough bread.</t>
+          <t>Bakery / Café in Berlin. Berlin-glutenfrei lists AERA Charlottenburg as vollständig glutenfreies Angebot and states that the bakery bakes exclusively gluten-free; AERA official site markets 100% gluten-free sourdough bread.</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>AERA is a fully gluten-free bakery/café in Berlin with a listed Mitte location; official brand source states 100% gluten-free sourdough bread.</t>
+          <t>Bakery / Café in Berlin. AERA is a fully gluten-free bakery/café in Berlin with a listed Mitte location; official brand source states 100% gluten-free sourdough bread.</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Official website states 100% gluten-free and natural; Berlin-glutenfrei states Oshione bakes exclusively gluten-free.</t>
+          <t>Bakery / Café in Berlin. Official website states 100% gluten-free and natural; Berlin-glutenfrei states Oshione bakes exclusively gluten-free.</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei states that Jute bakes exclusively gluten-free; the official impressum confirms the current business address.</t>
+          <t>Bakery / Café in Berlin. Berlin-glutenfrei states that Jute bakes exclusively gluten-free; the official impressum confirms the current business address.</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists it as vollständig glutenfreies Angebot and notes exclusively gluten-free products; only oat milk is handled separately.</t>
+          <t>Café / Breakfast / Brunch in Berlin. Berlin-glutenfrei lists it as vollständig glutenfreies Angebot and notes exclusively gluten-free products; only oat milk is handled separately.</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>Official website states baked goods are made exclusively gluten-free and vegan; Berlin-glutenfrei lists fully gluten-free offer.</t>
+          <t>Café / Bakery in Berlin. Official website states baked goods are made exclusively gluten-free and vegan; Berlin-glutenfrei lists fully gluten-free offer.</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei states all dishes are gluten-free; the official website/impressum confirms the current address.</t>
+          <t>Brazilian Restaurant / Café in Berlin. Berlin-glutenfrei states all dishes are gluten-free; the official website/impressum confirms the current address.</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei describes Trattoria Senza as a vollständig glutenfreies und lactosefreies Restaurant.</t>
+          <t>Restaurant / Italian in Berlin. Berlin-glutenfrei describes Trattoria Senza as a vollständig glutenfreies und lactosefreies Restaurant.</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei says everything is 100% gluten-free and safe for coeliacs; address is listed.</t>
+          <t>Café / Bakery in Berlin. Berlin-glutenfrei says everything is 100% gluten-free and safe for coeliacs; address is listed.</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists fully gluten-free offer and states that Pretty Hill bakes exclusively gluten-free.</t>
+          <t>Café / Bakery / Ice cream in Berlin. Berlin-glutenfrei lists fully gluten-free offer and states that Pretty Hill bakes exclusively gluten-free.</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists fully gluten-free offer and states all dishes are vegan, lactose-free and gluten-free.</t>
+          <t>Restaurant / Greek in Berlin. Berlin-glutenfrei lists fully gluten-free offer and states all dishes are vegan, lactose-free and gluten-free.</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists Café Prana under fully gluten-free bakery/café offers; Berlin Vegan confirms address.</t>
+          <t>Café / Bakery in Berlin. Berlin-glutenfrei lists Café Prana under fully gluten-free bakery/café offers; Berlin Vegan confirms address.</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>Isabella lists Hamburg–Alter Wall as an official gluten-free café; location pages state the bakery bakes exclusively gluten-free.</t>
+          <t>Bakery / Café / Pâtisserie in Hamburg. Isabella lists Hamburg–Alter Wall as an official gluten-free café; location pages state the bakery bakes exclusively gluten-free.</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>Official site states products are exclusively gluten-free and a dedicated page says the bakery works exclusively with gluten-free products so no contamination occurs.</t>
+          <t>Café / Bakery / Pastry in Hamburg. Official site states products are exclusively gluten-free and a dedicated page says the bakery works exclusively with gluten-free products so no contamination occurs.</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>Official website focuses on gluten-free breads; specialist sources classify the bakery as 100% gluten-free/dedicated; address confirmed via Gluto/Atly.</t>
+          <t>Bakery / Café in Hamburg. Official website focuses on gluten-free breads; specialist sources classify the bakery as 100% gluten-free/dedicated; address confirmed via Gluto/Atly.</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>Official Munich location page confirms Hackenstraße 4 and Isabella pages state gluten-free/certified gluten-free products; external listings describe 100% gluten-free offer.</t>
+          <t>Bakery / Café / Pâtisserie in München. Official Munich location page confirms Hackenstraße 4 and Isabella pages state gluten-free/certified gluten-free products; external listings describe 100% gluten-free offer.</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>Official direct-sale page says 100% glutenfrei &amp; bio at the Munich address; official Facebook also brands as 100% glutenfrei.</t>
+          <t>Bakery / Direct sale / Click &amp; Collect in München. Official direct-sale page says 100% glutenfrei &amp; bio at the Munich address; official Facebook also brands as 100% glutenfrei.</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>Official Instagram states 100% glutenfrei, vegan; local sources confirm address Barer Straße 48.</t>
+          <t>Café / Bakery / Community Space in München. Official Instagram states 100% glutenfrei, vegan; local sources confirm address Barer Straße 48.</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>Official website advertises 100% gluten-free food, beer and desserts and identifies a gluten-free kitchen.</t>
+          <t>Restaurant / Pizzeria / Paninoteca / Café in München. Official website advertises 100% gluten-free food, beer and desserts and identifies a gluten-free kitchen.</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>Isabella official café list includes Köln–Kettengasse; external location sources confirm address and 100% gluten-free positioning.</t>
+          <t>Bakery / Café / Pâtisserie in Köln. Isabella official café list includes Köln–Kettengasse; external location sources confirm address and 100% gluten-free positioning.</t>
         </is>
       </c>
       <c r="AF26" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>Atly lists the café as 100% dedicated gluten-free; Cologne guides describe that everything is gluten-free, lactose-free and without refined sugar.</t>
+          <t>Café / Raw cakes / Healthy sweets in Köln. Atly lists the café as 100% dedicated gluten-free; Cologne guides describe that everything is gluten-free, lactose-free and without refined sugar.</t>
         </is>
       </c>
       <c r="AF27" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>Official Isabella site lists gluten-free café location in Aachen; Isabella profile is 100% glutenfree brand.</t>
+          <t>Café / Pâtisserie in Aachen. Official Isabella site lists gluten-free café location in Aachen; Isabella profile is 100% glutenfree brand.</t>
         </is>
       </c>
       <c r="AF28" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="AE29" t="inlineStr">
         <is>
-          <t>Official Isabella café location; brand states gluten-free cafés and products.</t>
+          <t>Café / Pâtisserie in Düsseldorf. Official Isabella café location; brand states gluten-free cafés and products.</t>
         </is>
       </c>
       <c r="AF29" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="AE30" t="inlineStr">
         <is>
-          <t>Official Isabella to-go shop in Kö-Galerie; brand states gluten-free cafés/products.</t>
+          <t>To-go / Pâtisserie in Düsseldorf. Official Isabella to-go shop in Kö-Galerie; brand states gluten-free cafés/products.</t>
         </is>
       </c>
       <c r="AF30" t="inlineStr">
@@ -5129,7 +5129,7 @@
       </c>
       <c r="AE31" t="inlineStr">
         <is>
-          <t>Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Café / Pâtisserie in Stuttgart. Official Isabella location; gluten-free café/patisserie.</t>
         </is>
       </c>
       <c r="AF31" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="AE32" t="inlineStr">
         <is>
-          <t>Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Café / Pâtisserie in Stuttgart. Official Isabella location; gluten-free café/patisserie.</t>
         </is>
       </c>
       <c r="AF32" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="AE33" t="inlineStr">
         <is>
-          <t>Official website states entire product range is 100% gluten-free.</t>
+          <t>Bakery / Café in Düsseldorf. Official website states entire product range is 100% gluten-free.</t>
         </is>
       </c>
       <c r="AF33" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="AE34" t="inlineStr">
         <is>
-          <t>Official site states all food remains gluten-free; company profile says entire café/bistro offer is gluten-free.</t>
+          <t>Café / Bistro in Düsseldorf. Official site states all food remains gluten-free; company profile says entire café/bistro offer is gluten-free.</t>
         </is>
       </c>
       <c r="AF34" t="inlineStr">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="AE35" t="inlineStr">
         <is>
-          <t>Kiel Magazin describes backstube, café and pizzeria under one roof as 100% gluten-free and daily baked exclusively gluten-free.</t>
+          <t>Bakery / Café / Pizzeria in Kiel. Kiel Magazin describes backstube, café and pizzeria under one roof as 100% gluten-free and daily baked exclusively gluten-free.</t>
         </is>
       </c>
       <c r="AF35" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="AE36" t="inlineStr">
         <is>
-          <t>Official website states bio and 100% gluten-free; product pages state all products are 100% gluten-free.</t>
+          <t>Café / Bakery in Ettlingen. Official website states bio and 100% gluten-free; product pages state all products are 100% gluten-free.</t>
         </is>
       </c>
       <c r="AF36" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="AE37" t="inlineStr">
         <is>
-          <t>Official website states 100% gluten-free, no cross-contamination and gives physical shop/café address.</t>
+          <t>Bakery / Café / Shop in Freilassing. Official website states 100% gluten-free, no cross-contamination and gives physical shop/café address.</t>
         </is>
       </c>
       <c r="AF37" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="AE38" t="inlineStr">
         <is>
-          <t>Official Maisterei site describes 100% gluten-free bakery and café directly at the bakery.</t>
+          <t>Café / Bakery in Wetzlar. Official Maisterei site describes 100% gluten-free bakery and café directly at the bakery.</t>
         </is>
       </c>
       <c r="AF38" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="AE39" t="inlineStr">
         <is>
-          <t>Official website/Eatbu state all dishes are 100% gluten-free; restaurant and ordering profile active.</t>
+          <t>Restaurant / Pizzeria in Kassel. Official website/Eatbu state all dishes are 100% gluten-free; restaurant and ordering profile active.</t>
         </is>
       </c>
       <c r="AF39" t="inlineStr">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="AE40" t="inlineStr">
         <is>
-          <t>Official site brands 100% ohne Gluten; HNA reports all dishes are gluten-free at the newly opened restaurant.</t>
+          <t>Restaurant / Café / Bar in Kassel. Official site brands 100% ohne Gluten; HNA reports all dishes are gluten-free at the newly opened restaurant.</t>
         </is>
       </c>
       <c r="AF40" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="AE41" t="inlineStr">
         <is>
-          <t>Official website states all dishes are served guaranteed gluten-free and without glutamate.</t>
+          <t>Japanese / Sushi restaurant in Kassel. Official website states all dishes are served guaranteed gluten-free and without glutamate.</t>
         </is>
       </c>
       <c r="AF41" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AE42" t="inlineStr">
         <is>
-          <t>Official menu says the Vivarepas concept is completely gluten-free.</t>
+          <t>Restaurant in Pforzheim. Official menu says the Vivarepas concept is completely gluten-free.</t>
         </is>
       </c>
       <c r="AF42" t="inlineStr">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="AE43" t="inlineStr">
         <is>
-          <t>Official Instagram describes 100% plant-based, gluten-free, sugar-free cuisine; specialized sources also mark as completely GF.</t>
+          <t>Restaurant in Stuttgart. Official Instagram describes 100% plant-based, gluten-free, sugar-free cuisine; specialized sources also mark as completely GF.</t>
         </is>
       </c>
       <c r="AF43" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="AE44" t="inlineStr">
         <is>
-          <t>Official site presents gluten-free café; third-party coeliac sources mark it 100% dedicated GF. Use as publish, with owner recheck recommended before live badge.</t>
+          <t>Café / Concept Store in Brühl. Official site presents gluten-free café; third-party coeliac sources mark it 100% dedicated GF. Use as publish, with owner recheck recommended before live badge.</t>
         </is>
       </c>
       <c r="AF44" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="AE45" t="inlineStr">
         <is>
-          <t>City listing states Arepas, Empanadas and Bowls are all gluten-free; Atly labels location 100% dedicated GF.</t>
+          <t>Café / Coffee roastery in Heidelberg. City listing states Arepas, Empanadas and Bowls are all gluten-free; Atly labels location 100% dedicated GF.</t>
         </is>
       </c>
       <c r="AF45" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="AE46" t="inlineStr">
         <is>
-          <t>Official Facebook profile states café is 100% gluten-free and all food/drinks are suitable for coeliacs.</t>
+          <t>Café in Viernheim. Official Facebook profile states café is 100% gluten-free and all food/drinks are suitable for coeliacs.</t>
         </is>
       </c>
       <c r="AF46" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>Official Instagram name and posts brand the business as 100% gluten-free; no full website found, so owner confirmation recommended.</t>
+          <t>Pizzeria in Eisenach. Official Instagram name and posts brand the business as 100% gluten-free; no full website found, so owner confirmation recommended.</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
@@ -7492,7 +7492,7 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>Reviews and directories state the kitchen cooks/bakes exclusively gluten-free; no strong official website found, so owner confirmation recommended.</t>
+          <t>Restaurant / Pizzeria in Balingen. Reviews and directories state the kitchen cooks/bakes exclusively gluten-free; no strong official website found, so owner confirmation recommended.</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="AE49" t="inlineStr">
         <is>
-          <t>Atly marks Flora Café as 100% dedicated GF; community sources mention only gluten-free baking/cakes. Owner confirmation recommended before live badge.</t>
+          <t>Café in Fehmarn. Atly marks Flora Café as 100% dedicated GF; community sources mention only gluten-free baking/cakes. Owner confirmation recommended before live badge.</t>
         </is>
       </c>
       <c r="AF49" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>Official FAQ lists Hofladen/Gastronomie and answers that products are gluten-free; validate full gastronomy scope before live badge.</t>
+          <t>Bistro / Bakery / Hofladen in Bad Dürkheim. Official FAQ lists Hofladen/Gastronomie and answers that products are gluten-free; validate full gastronomy scope before live badge.</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="AE51" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; local/social sources state all food gluten- and lactose-free. Official website/owner confirmation recommended.</t>
+          <t>Restaurant in Regensburg. Atly marks 100% dedicated GF; local/social sources state all food gluten- and lactose-free. Official website/owner confirmation recommended.</t>
         </is>
       </c>
       <c r="AF51" t="inlineStr">
@@ -8048,7 +8048,7 @@
       </c>
       <c r="AE52" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; Reddit/community mentions 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Restaurant / Crêpes / Streetfood in Kamp-Lintfort. Atly marks 100% dedicated GF; Reddit/community mentions 100% GF. No official website found; owner confirmation required before live.</t>
         </is>
       </c>
       <c r="AF52" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="AE53" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; community mention says 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Café in Brüggen. Atly marks 100% dedicated GF; community mention says 100% GF. No official website found; owner confirmation required before live.</t>
         </is>
       </c>
       <c r="AF53" t="inlineStr">

</xml_diff>

<commit_message>
Update German restaurant descriptions from ES/DE copy deck.
Replace verification-focused blurbs with natural venue descriptions for 181 locations.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
+++ b/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
@@ -828,7 +828,7 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Café / Pâtisserie / Bakery in Frankfurt am Main. Official source states the bakery bakes exclusively gluten-free; Frankfurt location and address are listed on official site.</t>
+          <t>Bäckerei/Patisserie in Frankfurt am Main mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Restaurant / Vietnamese in Frankfurt am Main. Official site positions the restaurant with gluten-free branding and address; specialist/current community sources describe it as 100% gluten-free. Direct written confirmation still recommended for app maximum assurance.</t>
+          <t>Restaurant/Bistro in Frankfurt am Main mit Vorspeisen, Hauptgerichten, Desserts und je nach Konzept regionaler, mediterraner oder internationaler Küche.</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Café / Bakery / Raw cakes in Frankfurt am Main. Official site lists current address; Zöliakie Austausch states everything is 100% gluten-free. Old sources list Lindley/Oederweg, so location list must be rechecked before import.</t>
+          <t>Veganes bzw. plant-based Café/Restaurant in Frankfurt am Main mit Bowls, Kuchen, Frühstücksgerichten, Snacks und kreativer pflanzlicher Küche.</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Café / Bakery / Brunch in Frankfurt am Main. Current operator states she took over Kaffeebar by Alex and offers gluten-free specialties; legacy sources describe the location as completely gluten-free. Current official wording says gluten-free specialties/options, so direct confirmation recommended before hard 100%-GF badge.</t>
+          <t>Bäckerei/Patisserie in Frankfurt am Main mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Café / Superfood / Bowls in Bad Homburg vor der Höhe. Accepted for import as Frankfurt Rhein-Main / Bad Homburg. Official site describes a gluten-free café/products; specialist source says all products are gluten-free. City is Bad Homburg, not Frankfurt am Main, so region/city filters must show it as Bad Homburg.</t>
+          <t>Healthy-Restaurant/Café in Bad Homburg vor der Höhe mit Bowls, Brunchgerichten, Salaten, herzhaften Speisen, Kuchen und Getränken.</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Bakery / Café in Berlin. Berlin-glutenfrei lists AERA Charlottenburg as vollständig glutenfreies Angebot and states that the bakery bakes exclusively gluten-free; AERA official site markets 100% gluten-free sourdough bread.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Bakery / Café in Berlin. AERA is a fully gluten-free bakery/café in Berlin with a listed Mitte location; official brand source states 100% gluten-free sourdough bread.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Bakery / Café in Berlin. Official website states 100% gluten-free and natural; Berlin-glutenfrei states Oshione bakes exclusively gluten-free.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Bakery / Café in Berlin. Berlin-glutenfrei states that Jute bakes exclusively gluten-free; the official impressum confirms the current business address.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>Café / Breakfast / Brunch in Berlin. Berlin-glutenfrei lists it as vollständig glutenfreies Angebot and notes exclusively gluten-free products; only oat milk is handled separately.</t>
+          <t>Café in Berlin mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>Café / Bakery in Berlin. Official website states baked goods are made exclusively gluten-free and vegan; Berlin-glutenfrei lists fully gluten-free offer.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Brazilian Restaurant / Café in Berlin. Berlin-glutenfrei states all dishes are gluten-free; the official website/impressum confirms the current address.</t>
+          <t>Lateinamerikanisches Restaurant/Café in Berlin mit Tapioca, Arepas, Empanadas, Bowls und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>Restaurant / Italian in Berlin. Berlin-glutenfrei describes Trattoria Senza as a vollständig glutenfreies und lactosefreies Restaurant.</t>
+          <t>Italienisches Restaurant in Berlin mit Pizza, Pasta, Antipasti und weiteren mediterranen Gerichten.</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Café / Bakery in Berlin. Berlin-glutenfrei says everything is 100% gluten-free and safe for coeliacs; address is listed.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>Café / Bakery / Ice cream in Berlin. Berlin-glutenfrei lists fully gluten-free offer and states that Pretty Hill bakes exclusively gluten-free.</t>
+          <t>Veganes bzw. plant-based Café/Restaurant in Berlin mit Bowls, Kuchen, Frühstücksgerichten, Snacks und kreativer pflanzlicher Küche.</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>Restaurant / Greek in Berlin. Berlin-glutenfrei lists fully gluten-free offer and states all dishes are vegan, lactose-free and gluten-free.</t>
+          <t>Restaurant/Bistro in Berlin mit Vorspeisen, Hauptgerichten, Desserts und je nach Konzept regionaler, mediterraner oder internationaler Küche.</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>Café / Bakery in Berlin. Berlin-glutenfrei lists Café Prana under fully gluten-free bakery/café offers; Berlin Vegan confirms address.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>Bakery / Café / Pâtisserie in Hamburg. Isabella lists Hamburg–Alter Wall as an official gluten-free café; location pages state the bakery bakes exclusively gluten-free.</t>
+          <t>Bäckerei/Patisserie in Hamburg mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>Café / Bakery / Pastry in Hamburg. Official site states products are exclusively gluten-free and a dedicated page says the bakery works exclusively with gluten-free products so no contamination occurs.</t>
+          <t>Bäckerei/Patisserie in Hamburg mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>Bakery / Café in Hamburg. Official website focuses on gluten-free breads; specialist sources classify the bakery as 100% gluten-free/dedicated; address confirmed via Gluto/Atly.</t>
+          <t>Healthy-Restaurant/Café in Hamburg mit Bowls, Brunchgerichten, Salaten, herzhaften Speisen, Kuchen und Getränken.</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>Bakery / Café / Pâtisserie in München. Official Munich location page confirms Hackenstraße 4 and Isabella pages state gluten-free/certified gluten-free products; external listings describe 100% gluten-free offer.</t>
+          <t>Bäckerei/Patisserie in München mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>Bakery / Direct sale / Click &amp; Collect in München. Official direct-sale page says 100% glutenfrei &amp; bio at the Munich address; official Facebook also brands as 100% glutenfrei.</t>
+          <t>Bäckerei/Patisserie in München mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>Café / Bakery / Community Space in München. Official Instagram states 100% glutenfrei, vegan; local sources confirm address Barer Straße 48.</t>
+          <t>Veganes bzw. plant-based Café/Restaurant in München mit Bowls, Kuchen, Frühstücksgerichten, Snacks und kreativer pflanzlicher Küche.</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>Restaurant / Pizzeria / Paninoteca / Café in München. Official website advertises 100% gluten-free food, beer and desserts and identifies a gluten-free kitchen.</t>
+          <t>Pizzeria in München mit Pizza, herzhaften Ofengerichten und italienisch inspirierten Speisen.</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>Bakery / Café / Pâtisserie in Köln. Isabella official café list includes Köln–Kettengasse; external location sources confirm address and 100% gluten-free positioning.</t>
+          <t>Bäckerei/Patisserie in Köln mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF26" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>Café / Raw cakes / Healthy sweets in Köln. Atly lists the café as 100% dedicated gluten-free; Cologne guides describe that everything is gluten-free, lactose-free and without refined sugar.</t>
+          <t>Café in Köln mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF27" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>Café / Pâtisserie in Aachen. Official Isabella site lists gluten-free café location in Aachen; Isabella profile is 100% glutenfree brand.</t>
+          <t>Bäckerei/Patisserie in Aachen mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF28" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="AE29" t="inlineStr">
         <is>
-          <t>Café / Pâtisserie in Düsseldorf. Official Isabella café location; brand states gluten-free cafés and products.</t>
+          <t>Bäckerei/Patisserie in Düsseldorf mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF29" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="AE30" t="inlineStr">
         <is>
-          <t>To-go / Pâtisserie in Düsseldorf. Official Isabella to-go shop in Kö-Galerie; brand states gluten-free cafés/products.</t>
+          <t>Bäckerei/Patisserie in Düsseldorf mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF30" t="inlineStr">
@@ -5129,7 +5129,7 @@
       </c>
       <c r="AE31" t="inlineStr">
         <is>
-          <t>Café / Pâtisserie in Stuttgart. Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Bäckerei/Patisserie in Stuttgart mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF31" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="AE32" t="inlineStr">
         <is>
-          <t>Café / Pâtisserie in Stuttgart. Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Bäckerei/Patisserie in Stuttgart mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF32" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="AE33" t="inlineStr">
         <is>
-          <t>Bakery / Café in Düsseldorf. Official website states entire product range is 100% gluten-free.</t>
+          <t>Bäckerei/Patisserie in Düsseldorf mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF33" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="AE34" t="inlineStr">
         <is>
-          <t>Café / Bistro in Düsseldorf. Official site states all food remains gluten-free; company profile says entire café/bistro offer is gluten-free.</t>
+          <t>Café in Düsseldorf mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF34" t="inlineStr">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="AE35" t="inlineStr">
         <is>
-          <t>Bakery / Café / Pizzeria in Kiel. Kiel Magazin describes backstube, café and pizzeria under one roof as 100% gluten-free and daily baked exclusively gluten-free.</t>
+          <t>Pizzeria in Kiel mit Pizza, herzhaften Ofengerichten und italienisch inspirierten Speisen.</t>
         </is>
       </c>
       <c r="AF35" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="AE36" t="inlineStr">
         <is>
-          <t>Café / Bakery in Ettlingen. Official website states bio and 100% gluten-free; product pages state all products are 100% gluten-free.</t>
+          <t>Bäckerei/Patisserie in Ettlingen mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF36" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="AE37" t="inlineStr">
         <is>
-          <t>Bakery / Café / Shop in Freilassing. Official website states 100% gluten-free, no cross-contamination and gives physical shop/café address.</t>
+          <t>Bäckerei/Patisserie in Freilassing mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF37" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="AE38" t="inlineStr">
         <is>
-          <t>Café / Bakery in Wetzlar. Official Maisterei site describes 100% gluten-free bakery and café directly at the bakery.</t>
+          <t>Bäckerei/Patisserie in Wetzlar mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF38" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="AE39" t="inlineStr">
         <is>
-          <t>Restaurant / Pizzeria in Kassel. Official website/Eatbu state all dishes are 100% gluten-free; restaurant and ordering profile active.</t>
+          <t>Pizzeria in Kassel mit Pizza, herzhaften Ofengerichten und italienisch inspirierten Speisen.</t>
         </is>
       </c>
       <c r="AF39" t="inlineStr">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="AE40" t="inlineStr">
         <is>
-          <t>Restaurant / Café / Bar in Kassel. Official site brands 100% ohne Gluten; HNA reports all dishes are gluten-free at the newly opened restaurant.</t>
+          <t>Café in Kassel mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF40" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="AE41" t="inlineStr">
         <is>
-          <t>Japanese / Sushi restaurant in Kassel. Official website states all dishes are served guaranteed gluten-free and without glutamate.</t>
+          <t>Japanisches Restaurant in Kassel mit Sushi, warmen japanischen Gerichten, Reisgerichten und Desserts.</t>
         </is>
       </c>
       <c r="AF41" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AE42" t="inlineStr">
         <is>
-          <t>Restaurant in Pforzheim. Official menu says the Vivarepas concept is completely gluten-free.</t>
+          <t>Lateinamerikanisches Restaurant/Café in Pforzheim mit Tapioca, Arepas, Empanadas, Bowls und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF42" t="inlineStr">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="AE43" t="inlineStr">
         <is>
-          <t>Restaurant in Stuttgart. Official Instagram describes 100% plant-based, gluten-free, sugar-free cuisine; specialized sources also mark as completely GF.</t>
+          <t>Veganes bzw. plant-based Café/Restaurant in Stuttgart mit Bowls, Kuchen, Frühstücksgerichten, Snacks und kreativer pflanzlicher Küche.</t>
         </is>
       </c>
       <c r="AF43" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="AE44" t="inlineStr">
         <is>
-          <t>Café / Concept Store in Brühl. Official site presents gluten-free café; third-party coeliac sources mark it 100% dedicated GF. Use as publish, with owner recheck recommended before live badge.</t>
+          <t>Café in Brühl mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF44" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="AE45" t="inlineStr">
         <is>
-          <t>Café / Coffee roastery in Heidelberg. City listing states Arepas, Empanadas and Bowls are all gluten-free; Atly labels location 100% dedicated GF.</t>
+          <t>Café in Heidelberg mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF45" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="AE46" t="inlineStr">
         <is>
-          <t>Café in Viernheim. Official Facebook profile states café is 100% gluten-free and all food/drinks are suitable for coeliacs.</t>
+          <t>Café in Viernheim mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF46" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>Pizzeria in Eisenach. Official Instagram name and posts brand the business as 100% gluten-free; no full website found, so owner confirmation recommended.</t>
+          <t>Pizzeria in Eisenach mit Pizza, herzhaften Ofengerichten und italienisch inspirierten Speisen.</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
@@ -7492,7 +7492,7 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>Restaurant / Pizzeria in Balingen. Reviews and directories state the kitchen cooks/bakes exclusively gluten-free; no strong official website found, so owner confirmation recommended.</t>
+          <t>Pizzeria in Balingen mit Pizza, herzhaften Ofengerichten und italienisch inspirierten Speisen.</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="AE49" t="inlineStr">
         <is>
-          <t>Café in Fehmarn. Atly marks Flora Café as 100% dedicated GF; community sources mention only gluten-free baking/cakes. Owner confirmation recommended before live badge.</t>
+          <t>Café in Fehmarn mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF49" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>Bistro / Bakery / Hofladen in Bad Dürkheim. Official FAQ lists Hofladen/Gastronomie and answers that products are gluten-free; validate full gastronomy scope before live badge.</t>
+          <t>Bäckerei/Patisserie in Bad Dürkheim mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="AE51" t="inlineStr">
         <is>
-          <t>Restaurant in Regensburg. Atly marks 100% dedicated GF; local/social sources state all food gluten- and lactose-free. Official website/owner confirmation recommended.</t>
+          <t>Restaurant/Bistro in Regensburg mit Vorspeisen, Hauptgerichten, Desserts und je nach Konzept regionaler, mediterraner oder internationaler Küche.</t>
         </is>
       </c>
       <c r="AF51" t="inlineStr">
@@ -8048,7 +8048,7 @@
       </c>
       <c r="AE52" t="inlineStr">
         <is>
-          <t>Restaurant / Crêpes / Streetfood in Kamp-Lintfort. Atly marks 100% dedicated GF; Reddit/community mentions 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Restaurant/Bistro in Kamp-Lintfort mit Vorspeisen, Hauptgerichten, Desserts und je nach Konzept regionaler, mediterraner oder internationaler Küche.</t>
         </is>
       </c>
       <c r="AF52" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="AE53" t="inlineStr">
         <is>
-          <t>Café in Brüggen. Atly marks 100% dedicated GF; community mention says 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Café in Brüggen mit Kaffee, Frühstück, Kuchen, Gebäck, Brunchgerichten und kleinen Speisen.</t>
         </is>
       </c>
       <c r="AF53" t="inlineStr">

</xml_diff>

<commit_message>
Normalize restaurant descriptions across DE, EN, and ES.
Replace audit-style copy and internal seed notes with natural template-based texts; all 190 venues now have descriptions in all three languages with localized city names.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
+++ b/data-source/CeliacSafe_Datenbank_v4_Germany_Delta_Consolidated_geocoded.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>Official source states the bakery bakes exclusively gluten-free; Frankfurt location and address are listed on official site.</t>
+          <t>Bakery and patisserie in Frankfurt am Main offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Official source states the bakery bakes exclusively gluten-free; Frankfurt location and address are listed on official site.</t>
+          <t>Panadería y pastelería en Fráncfort del Meno con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI2" t="b">
@@ -982,12 +982,12 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>Official site positions the restaurant with gluten-free branding and address; specialist/current community sources describe it as 100% gluten-free. Direct written confirmation still recommended for app maximum assurance.</t>
+          <t>Restaurant and bistro in Frankfurt am Main serving starters, main courses, and desserts, with regional, Mediterranean, or international cuisine depending on the concept.</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Official site positions the restaurant with gluten-free branding and address; specialist/current community sources describe it as 100% gluten-free. Direct written confirmation still recommended for app maximum assurance.</t>
+          <t>Restaurante y bistró en Fráncfort del Meno con entrantes, platos principales y postres; cocina regional, mediterránea o internacional según el concepto.</t>
         </is>
       </c>
       <c r="AI3" t="b">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>Official site lists current address; Zöliakie Austausch states everything is 100% gluten-free. Old sources list Lindley/Oederweg, so location list must be rechecked before import.</t>
+          <t>Vegan, plant-based café and restaurant in Frankfurt am Main offering bowls, cakes, breakfast dishes, snacks, and creative plant-based cuisine.</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Official site lists current address; Zöliakie Austausch states everything is 100% gluten-free. Old sources list Lindley/Oederweg, so location list must be rechecked before import.</t>
+          <t>Cafetería y restaurante vegano en Fráncfort del Meno con bowls, tartas, desayunos, snacks y cocina vegetal creativa.</t>
         </is>
       </c>
       <c r="AI4" t="b">
@@ -1280,12 +1280,12 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>Current operator states she took over Kaffeebar by Alex and offers gluten-free specialties; legacy sources describe the location as completely gluten-free. Current official wording says gluten-free specialties/options, so direct confirmation recommended before hard 100%-GF badge.</t>
+          <t>Bakery and patisserie in Frankfurt am Main offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Current operator states she took over Kaffeebar by Alex and offers gluten-free specialties; legacy sources describe the location as completely gluten-free. Current official wording says gluten-free specialties/options, so direct confirmation recommended before hard 100%-GF badge.</t>
+          <t>Panadería y pastelería en Fráncfort del Meno con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI5" t="b">
@@ -1429,12 +1429,12 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>Accepted for import as Frankfurt Rhein-Main / Bad Homburg. Official site describes a gluten-free café/products; specialist source says all products are gluten-free. City is Bad Homburg, not Frankfurt am Main, so region/city filters must show it as Bad Homburg.</t>
+          <t>Health-focused restaurant and café in Bad Homburg vor der Höhe offering bowls, brunch dishes, salads, savoury plates, cakes, and drinks.</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>Accepted for import as Frankfurt Rhein-Main / Bad Homburg. Official site describes a gluten-free café/products; specialist source says all products are gluten-free. City is Bad Homburg, not Frankfurt am Main, so region/city filters must show it as Bad Homburg.</t>
+          <t>Restaurante y cafetería saludable en Bad Homburg vor der Höhe con bowls, platos de brunch, ensaladas, platos salados, tartas y bebidas.</t>
         </is>
       </c>
       <c r="AI6" t="b">
@@ -1578,12 +1578,12 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists AERA Charlottenburg as vollständig glutenfreies Angebot and states that the bakery bakes exclusively gluten-free; AERA official site markets 100% gluten-free sourdough bread.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists AERA Charlottenburg as vollständig glutenfreies Angebot and states that the bakery bakes exclusively gluten-free; AERA official site markets 100% gluten-free sourdough bread.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI7" t="b">
@@ -1727,12 +1727,12 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>AERA is a fully gluten-free bakery/café in Berlin with a listed Mitte location; official brand source states 100% gluten-free sourdough bread.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>AERA is a fully gluten-free bakery/café in Berlin with a listed Mitte location; official brand source states 100% gluten-free sourdough bread.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI8" t="b">
@@ -1876,12 +1876,12 @@
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>Official website states 100% gluten-free and natural; Berlin-glutenfrei states Oshione bakes exclusively gluten-free.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Official website states 100% gluten-free and natural; Berlin-glutenfrei states Oshione bakes exclusively gluten-free.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI9" t="b">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei states that Jute bakes exclusively gluten-free; the official impressum confirms the current business address.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei states that Jute bakes exclusively gluten-free; the official impressum confirms the current business address.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI10" t="b">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists it as vollständig glutenfreies Angebot and notes exclusively gluten-free products; only oat milk is handled separately.</t>
+          <t>Café in Berlin offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists it as vollständig glutenfreies Angebot and notes exclusively gluten-free products; only oat milk is handled separately.</t>
+          <t>Cafetería en Berlín con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI11" t="b">
@@ -2328,12 +2328,12 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>Official website states baked goods are made exclusively gluten-free and vegan; Berlin-glutenfrei lists fully gluten-free offer.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Official website states baked goods are made exclusively gluten-free and vegan; Berlin-glutenfrei lists fully gluten-free offer.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI12" t="b">
@@ -2477,12 +2477,12 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei states all dishes are gluten-free; the official website/impressum confirms the current address.</t>
+          <t>Latin American restaurant and café in Berlin serving tapioca, arepas, empanadas, bowls, and savoury snacks.</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei states all dishes are gluten-free; the official website/impressum confirms the current address.</t>
+          <t>Restaurante y café latinoamericano en Berlín con tapioca, arepas, empanadas, bowls y snacks salados.</t>
         </is>
       </c>
       <c r="AI13" t="b">
@@ -2626,12 +2626,12 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei describes Trattoria Senza as a vollständig glutenfreies und lactosefreies Restaurant.</t>
+          <t>Italian restaurant in Berlin serving pizza, pasta, antipasti, and other Mediterranean dishes.</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei describes Trattoria Senza as a vollständig glutenfreies und lactosefreies Restaurant.</t>
+          <t>Restaurante italiano en Berlín con pizza, pasta, antipasti y otros platos mediterráneos.</t>
         </is>
       </c>
       <c r="AI14" t="b">
@@ -2785,12 +2785,12 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei says everything is 100% gluten-free and safe for coeliacs; address is listed.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei says everything is 100% gluten-free and safe for coeliacs; address is listed.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI15" t="b">
@@ -2934,12 +2934,12 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists fully gluten-free offer and states that Pretty Hill bakes exclusively gluten-free.</t>
+          <t>Vegan, plant-based café and restaurant in Berlin offering bowls, cakes, breakfast dishes, snacks, and creative plant-based cuisine.</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists fully gluten-free offer and states that Pretty Hill bakes exclusively gluten-free.</t>
+          <t>Cafetería y restaurante vegano en Berlín con bowls, tartas, desayunos, snacks y cocina vegetal creativa.</t>
         </is>
       </c>
       <c r="AI16" t="b">
@@ -3083,12 +3083,12 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists fully gluten-free offer and states all dishes are vegan, lactose-free and gluten-free.</t>
+          <t>Restaurant and bistro in Berlin serving starters, main courses, and desserts, with regional, Mediterranean, or international cuisine depending on the concept.</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists fully gluten-free offer and states all dishes are vegan, lactose-free and gluten-free.</t>
+          <t>Restaurante y bistró en Berlín con entrantes, platos principales y postres; cocina regional, mediterránea o internacional según el concepto.</t>
         </is>
       </c>
       <c r="AI17" t="b">
@@ -3232,12 +3232,12 @@
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists Café Prana under fully gluten-free bakery/café offers; Berlin Vegan confirms address.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Berlin-glutenfrei lists Café Prana under fully gluten-free bakery/café offers; Berlin Vegan confirms address.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI18" t="b">
@@ -3381,12 +3381,12 @@
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>Isabella lists Hamburg–Alter Wall as an official gluten-free café; location pages state the bakery bakes exclusively gluten-free.</t>
+          <t>Bakery and patisserie in Hamburg offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>Isabella lists Hamburg–Alter Wall as an official gluten-free café; location pages state the bakery bakes exclusively gluten-free.</t>
+          <t>Panadería y pastelería en Hamburgo con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI19" t="b">
@@ -3530,12 +3530,12 @@
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>Official site states products are exclusively gluten-free and a dedicated page says the bakery works exclusively with gluten-free products so no contamination occurs.</t>
+          <t>Bakery and patisserie in Hamburg offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>Official site states products are exclusively gluten-free and a dedicated page says the bakery works exclusively with gluten-free products so no contamination occurs.</t>
+          <t>Panadería y pastelería en Hamburgo con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI20" t="b">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>Official website focuses on gluten-free breads; specialist sources classify the bakery as 100% gluten-free/dedicated; address confirmed via Gluto/Atly.</t>
+          <t>Health-focused restaurant and café in Hamburg offering bowls, brunch dishes, salads, savoury plates, cakes, and drinks.</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>Official website focuses on gluten-free breads; specialist sources classify the bakery as 100% gluten-free/dedicated; address confirmed via Gluto/Atly.</t>
+          <t>Restaurante y cafetería saludable en Hamburgo con bowls, platos de brunch, ensaladas, platos salados, tartas y bebidas.</t>
         </is>
       </c>
       <c r="AI21" t="b">
@@ -3828,12 +3828,12 @@
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>Official Munich location page confirms Hackenstraße 4 and Isabella pages state gluten-free/certified gluten-free products; external listings describe 100% gluten-free offer.</t>
+          <t>Bakery and patisserie in Munich offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>Official Munich location page confirms Hackenstraße 4 and Isabella pages state gluten-free/certified gluten-free products; external listings describe 100% gluten-free offer.</t>
+          <t>Panadería y pastelería en Múnich con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI22" t="b">
@@ -3977,12 +3977,12 @@
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>Official direct-sale page says 100% glutenfrei &amp; bio at the Munich address; official Facebook also brands as 100% glutenfrei.</t>
+          <t>Bakery and patisserie in Munich offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>Official direct-sale page says 100% glutenfrei &amp; bio at the Munich address; official Facebook also brands as 100% glutenfrei.</t>
+          <t>Panadería y pastelería en Múnich con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI23" t="b">
@@ -4126,12 +4126,12 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>Official Instagram states 100% glutenfrei, vegan; local sources confirm address Barer Straße 48.</t>
+          <t>Vegan, plant-based café and restaurant in Munich offering bowls, cakes, breakfast dishes, snacks, and creative plant-based cuisine.</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>Official Instagram states 100% glutenfrei, vegan; local sources confirm address Barer Straße 48.</t>
+          <t>Cafetería y restaurante vegano en Múnich con bowls, tartas, desayunos, snacks y cocina vegetal creativa.</t>
         </is>
       </c>
       <c r="AI24" t="b">
@@ -4275,12 +4275,12 @@
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>Official website advertises 100% gluten-free food, beer and desserts and identifies a gluten-free kitchen.</t>
+          <t>Pizzeria in Munich serving pizza, savoury oven-baked dishes, and Italian-inspired food.</t>
         </is>
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>Official website advertises 100% gluten-free food, beer and desserts and identifies a gluten-free kitchen.</t>
+          <t>Pizzería en Múnich con pizza, platos al horno y cocina de inspiración italiana.</t>
         </is>
       </c>
       <c r="AI25" t="b">
@@ -4424,12 +4424,12 @@
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>Isabella official café list includes Köln–Kettengasse; external location sources confirm address and 100% gluten-free positioning.</t>
+          <t>Bakery and patisserie in Cologne offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>Isabella official café list includes Köln–Kettengasse; external location sources confirm address and 100% gluten-free positioning.</t>
+          <t>Panadería y pastelería en Colonia con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI26" t="b">
@@ -4573,12 +4573,12 @@
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>Atly lists the café as 100% dedicated gluten-free; Cologne guides describe that everything is gluten-free, lactose-free and without refined sugar.</t>
+          <t>Café in Cologne offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>Atly lists the café as 100% dedicated gluten-free; Cologne guides describe that everything is gluten-free, lactose-free and without refined sugar.</t>
+          <t>Cafetería en Colonia con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI27" t="b">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="AF28" t="inlineStr">
         <is>
-          <t>Official Isabella site lists gluten-free café location in Aachen; Isabella profile is 100% glutenfree brand.</t>
+          <t>Bakery and patisserie in Aachen offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG28" t="inlineStr">
         <is>
-          <t>Official Isabella site lists gluten-free café location in Aachen; Isabella profile is 100% glutenfree brand.</t>
+          <t>Panadería y pastelería en Aquisgrán con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI28" t="b">
@@ -4856,12 +4856,12 @@
       </c>
       <c r="AF29" t="inlineStr">
         <is>
-          <t>Official Isabella café location; brand states gluten-free cafés and products.</t>
+          <t>Bakery and patisserie in Düsseldorf offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG29" t="inlineStr">
         <is>
-          <t>Official Isabella café location; brand states gluten-free cafés and products.</t>
+          <t>Panadería y pastelería en Düsseldorf con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI29" t="b">
@@ -4995,12 +4995,12 @@
       </c>
       <c r="AF30" t="inlineStr">
         <is>
-          <t>Official Isabella to-go shop in Kö-Galerie; brand states gluten-free cafés/products.</t>
+          <t>Bakery and patisserie in Düsseldorf offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>Official Isabella to-go shop in Kö-Galerie; brand states gluten-free cafés/products.</t>
+          <t>Panadería y pastelería en Düsseldorf con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI30" t="b">
@@ -5134,12 +5134,12 @@
       </c>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Bakery and patisserie in Stuttgart offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG31" t="inlineStr">
         <is>
-          <t>Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Panadería y pastelería en Stuttgart con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI31" t="b">
@@ -5273,12 +5273,12 @@
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Bakery and patisserie in Stuttgart offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>Official Isabella location; gluten-free café/patisserie.</t>
+          <t>Panadería y pastelería en Stuttgart con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI32" t="b">
@@ -5412,12 +5412,12 @@
       </c>
       <c r="AF33" t="inlineStr">
         <is>
-          <t>Official website states entire product range is 100% gluten-free.</t>
+          <t>Bakery and patisserie in Düsseldorf offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>Official website states entire product range is 100% gluten-free.</t>
+          <t>Panadería y pastelería en Düsseldorf con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI33" t="b">
@@ -5551,12 +5551,12 @@
       </c>
       <c r="AF34" t="inlineStr">
         <is>
-          <t>Official site states all food remains gluten-free; company profile says entire café/bistro offer is gluten-free.</t>
+          <t>Café in Düsseldorf offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>Official site states all food remains gluten-free; company profile says entire café/bistro offer is gluten-free.</t>
+          <t>Cafetería en Düsseldorf con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI34" t="b">
@@ -5690,12 +5690,12 @@
       </c>
       <c r="AF35" t="inlineStr">
         <is>
-          <t>Kiel Magazin describes backstube, café and pizzeria under one roof as 100% gluten-free and daily baked exclusively gluten-free.</t>
+          <t>Pizzeria in Kiel serving pizza, savoury oven-baked dishes, and Italian-inspired food.</t>
         </is>
       </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>Kiel Magazin describes backstube, café and pizzeria under one roof as 100% gluten-free and daily baked exclusively gluten-free.</t>
+          <t>Pizzería en Kiel con pizza, platos al horno y cocina de inspiración italiana.</t>
         </is>
       </c>
       <c r="AI35" t="b">
@@ -5829,12 +5829,12 @@
       </c>
       <c r="AF36" t="inlineStr">
         <is>
-          <t>Official website states bio and 100% gluten-free; product pages state all products are 100% gluten-free.</t>
+          <t>Bakery and patisserie in Ettlingen offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>Official website states bio and 100% gluten-free; product pages state all products are 100% gluten-free.</t>
+          <t>Panadería y pastelería en Ettlingen con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI36" t="b">
@@ -5968,12 +5968,12 @@
       </c>
       <c r="AF37" t="inlineStr">
         <is>
-          <t>Official website states 100% gluten-free, no cross-contamination and gives physical shop/café address.</t>
+          <t>Bakery and patisserie in Freilassing offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>Official website states 100% gluten-free, no cross-contamination and gives physical shop/café address.</t>
+          <t>Panadería y pastelería en Freilassing con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI37" t="b">
@@ -6107,12 +6107,12 @@
       </c>
       <c r="AF38" t="inlineStr">
         <is>
-          <t>Official Maisterei site describes 100% gluten-free bakery and café directly at the bakery.</t>
+          <t>Bakery and patisserie in Wetzlar offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG38" t="inlineStr">
         <is>
-          <t>Official Maisterei site describes 100% gluten-free bakery and café directly at the bakery.</t>
+          <t>Panadería y pastelería en Wetzlar con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI38" t="b">
@@ -6246,12 +6246,12 @@
       </c>
       <c r="AF39" t="inlineStr">
         <is>
-          <t>Official website/Eatbu state all dishes are 100% gluten-free; restaurant and ordering profile active.</t>
+          <t>Pizzeria in Kassel serving pizza, savoury oven-baked dishes, and Italian-inspired food.</t>
         </is>
       </c>
       <c r="AG39" t="inlineStr">
         <is>
-          <t>Official website/Eatbu state all dishes are 100% gluten-free; restaurant and ordering profile active.</t>
+          <t>Pizzería en Kassel con pizza, platos al horno y cocina de inspiración italiana.</t>
         </is>
       </c>
       <c r="AI39" t="b">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="AF40" t="inlineStr">
         <is>
-          <t>Official site brands 100% ohne Gluten; HNA reports all dishes are gluten-free at the newly opened restaurant.</t>
+          <t>Café in Kassel offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG40" t="inlineStr">
         <is>
-          <t>Official site brands 100% ohne Gluten; HNA reports all dishes are gluten-free at the newly opened restaurant.</t>
+          <t>Cafetería en Kassel con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI40" t="b">
@@ -6524,12 +6524,12 @@
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>Official website states all dishes are served guaranteed gluten-free and without glutamate.</t>
+          <t>Japanese restaurant in Kassel serving sushi, hot Japanese dishes, rice dishes, and desserts.</t>
         </is>
       </c>
       <c r="AG41" t="inlineStr">
         <is>
-          <t>Official website states all dishes are served guaranteed gluten-free and without glutamate.</t>
+          <t>Restaurante japonés en Kassel con sushi, platos japoneses calientes, platos de arroz y postres.</t>
         </is>
       </c>
       <c r="AI41" t="b">
@@ -6663,12 +6663,12 @@
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>Official menu says the Vivarepas concept is completely gluten-free.</t>
+          <t>Latin American restaurant and café in Pforzheim serving tapioca, arepas, empanadas, bowls, and savoury snacks.</t>
         </is>
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>Official menu says the Vivarepas concept is completely gluten-free.</t>
+          <t>Restaurante y café latinoamericano en Pforzheim con tapioca, arepas, empanadas, bowls y snacks salados.</t>
         </is>
       </c>
       <c r="AI42" t="b">
@@ -6802,12 +6802,12 @@
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>Official Instagram describes 100% plant-based, gluten-free, sugar-free cuisine; specialized sources also mark as completely GF.</t>
+          <t>Vegan, plant-based café and restaurant in Stuttgart offering bowls, cakes, breakfast dishes, snacks, and creative plant-based cuisine.</t>
         </is>
       </c>
       <c r="AG43" t="inlineStr">
         <is>
-          <t>Official Instagram describes 100% plant-based, gluten-free, sugar-free cuisine; specialized sources also mark as completely GF.</t>
+          <t>Cafetería y restaurante vegano en Stuttgart con bowls, tartas, desayunos, snacks y cocina vegetal creativa.</t>
         </is>
       </c>
       <c r="AI43" t="b">
@@ -6941,12 +6941,12 @@
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>Official site presents gluten-free café; third-party coeliac sources mark it 100% dedicated GF. Use as publish, with owner recheck recommended before live badge.</t>
+          <t>Café in Brühl offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>Official site presents gluten-free café; third-party coeliac sources mark it 100% dedicated GF. Use as publish, with owner recheck recommended before live badge.</t>
+          <t>Cafetería en Brühl con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI44" t="b">
@@ -7080,12 +7080,12 @@
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>City listing states Arepas, Empanadas and Bowls are all gluten-free; Atly labels location 100% dedicated GF.</t>
+          <t>Café in Heidelberg offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>City listing states Arepas, Empanadas and Bowls are all gluten-free; Atly labels location 100% dedicated GF.</t>
+          <t>Cafetería en Heidelberg con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI45" t="b">
@@ -7219,12 +7219,12 @@
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>Official Facebook profile states café is 100% gluten-free and all food/drinks are suitable for coeliacs.</t>
+          <t>Café in Viernheim offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG46" t="inlineStr">
         <is>
-          <t>Official Facebook profile states café is 100% gluten-free and all food/drinks are suitable for coeliacs.</t>
+          <t>Cafetería en Viernheim con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI46" t="b">
@@ -7358,12 +7358,12 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>Official Instagram name and posts brand the business as 100% gluten-free; no full website found, so owner confirmation recommended.</t>
+          <t>Pizzeria in Eisenach serving pizza, savoury oven-baked dishes, and Italian-inspired food.</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>Official Instagram name and posts brand the business as 100% gluten-free; no full website found, so owner confirmation recommended.</t>
+          <t>Pizzería en Eisenach con pizza, platos al horno y cocina de inspiración italiana.</t>
         </is>
       </c>
       <c r="AI47" t="b">
@@ -7497,12 +7497,12 @@
       </c>
       <c r="AF48" t="inlineStr">
         <is>
-          <t>Reviews and directories state the kitchen cooks/bakes exclusively gluten-free; no strong official website found, so owner confirmation recommended.</t>
+          <t>Pizzeria in Balingen serving pizza, savoury oven-baked dishes, and Italian-inspired food.</t>
         </is>
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>Reviews and directories state the kitchen cooks/bakes exclusively gluten-free; no strong official website found, so owner confirmation recommended.</t>
+          <t>Pizzería en Balingen con pizza, platos al horno y cocina de inspiración italiana.</t>
         </is>
       </c>
       <c r="AI48" t="b">
@@ -7636,12 +7636,12 @@
       </c>
       <c r="AF49" t="inlineStr">
         <is>
-          <t>Atly marks Flora Café as 100% dedicated GF; community sources mention only gluten-free baking/cakes. Owner confirmation recommended before live badge.</t>
+          <t>Café in Fehmarn offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>Atly marks Flora Café as 100% dedicated GF; community sources mention only gluten-free baking/cakes. Owner confirmation recommended before live badge.</t>
+          <t>Cafetería en Fehmarn con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI49" t="b">
@@ -7775,12 +7775,12 @@
       </c>
       <c r="AF50" t="inlineStr">
         <is>
-          <t>Official FAQ lists Hofladen/Gastronomie and answers that products are gluten-free; validate full gastronomy scope before live badge.</t>
+          <t>Bakery and patisserie in Bad Dürkheim offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>Official FAQ lists Hofladen/Gastronomie and answers that products are gluten-free; validate full gastronomy scope before live badge.</t>
+          <t>Panadería y pastelería en Bad Dürkheim con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI50" t="b">
@@ -7914,12 +7914,12 @@
       </c>
       <c r="AF51" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; local/social sources state all food gluten- and lactose-free. Official website/owner confirmation recommended.</t>
+          <t>Restaurant and bistro in Regensburg serving starters, main courses, and desserts, with regional, Mediterranean, or international cuisine depending on the concept.</t>
         </is>
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; local/social sources state all food gluten- and lactose-free. Official website/owner confirmation recommended.</t>
+          <t>Restaurante y bistró en Ratisbona con entrantes, platos principales y postres; cocina regional, mediterránea o internacional según el concepto.</t>
         </is>
       </c>
       <c r="AI51" t="b">
@@ -8053,12 +8053,12 @@
       </c>
       <c r="AF52" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; Reddit/community mentions 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Restaurant and bistro in Kamp-Lintfort serving starters, main courses, and desserts, with regional, Mediterranean, or international cuisine depending on the concept.</t>
         </is>
       </c>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; Reddit/community mentions 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Restaurante y bistró en Kamp-Lintfort con entrantes, platos principales y postres; cocina regional, mediterránea o internacional según el concepto.</t>
         </is>
       </c>
       <c r="AI52" t="b">
@@ -8192,12 +8192,12 @@
       </c>
       <c r="AF53" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; community mention says 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Café in Brüggen offering coffee, breakfast, cakes, pastries, brunch dishes, and light bites.</t>
         </is>
       </c>
       <c r="AG53" t="inlineStr">
         <is>
-          <t>Atly marks 100% dedicated GF; community mention says 100% GF. No official website found; owner confirmation required before live.</t>
+          <t>Cafetería en Brüggen con café, desayunos, tartas, bollería, platos de brunch y comidas ligeras.</t>
         </is>
       </c>
       <c r="AI53" t="b">
@@ -8346,17 +8346,17 @@
       </c>
       <c r="AE54" t="inlineStr">
         <is>
-          <t>AERA Bread Charlottenburg ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF54" t="inlineStr">
         <is>
-          <t>AERA Bread Charlottenburg is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>AERA Bread Charlottenburg es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI54" t="b">
@@ -8575,17 +8575,17 @@
       </c>
       <c r="AE55" t="inlineStr">
         <is>
-          <t>AERA Bread Mitte ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF55" t="inlineStr">
         <is>
-          <t>AERA Bread Mitte is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>AERA Bread Mitte es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI55" t="b">
@@ -8804,17 +8804,17 @@
       </c>
       <c r="AE56" t="inlineStr">
         <is>
-          <t>Oshione Kreuzberg / Schöneberg ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF56" t="inlineStr">
         <is>
-          <t>Oshione Kreuzberg / Schöneberg is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG56" t="inlineStr">
         <is>
-          <t>Oshione Kreuzberg / Schöneberg es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI56" t="b">
@@ -9033,17 +9033,17 @@
       </c>
       <c r="AE57" t="inlineStr">
         <is>
-          <t>Oshione Neukölln / Weichselstraße ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Berlin mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF57" t="inlineStr">
         <is>
-          <t>Oshione Neukölln / Weichselstraße is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Berlin offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG57" t="inlineStr">
         <is>
-          <t>Oshione Neukölln / Weichselstraße es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Berlín con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI57" t="b">
@@ -9267,17 +9267,17 @@
       </c>
       <c r="AE58" t="inlineStr">
         <is>
-          <t>Backbrüder Essen ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Essen mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF58" t="inlineStr">
         <is>
-          <t>Backbrüder Essen is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Essen offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG58" t="inlineStr">
         <is>
-          <t>Backbrüder Essen es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Essen con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI58" t="b">
@@ -9501,17 +9501,17 @@
       </c>
       <c r="AE59" t="inlineStr">
         <is>
-          <t>Backbrüder Düsseldorf ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Düsseldorf mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF59" t="inlineStr">
         <is>
-          <t>Backbrüder Düsseldorf is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Düsseldorf offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG59" t="inlineStr">
         <is>
-          <t>Backbrüder Düsseldorf es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Düsseldorf con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI59" t="b">
@@ -9735,17 +9735,17 @@
       </c>
       <c r="AE60" t="inlineStr">
         <is>
-          <t>Plants &amp; Cakes Store ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Veganes bzw. plant-based Café/Restaurant in Frankfurt am Main mit Bowls, Kuchen, Frühstücksgerichten, Snacks und kreativer pflanzlicher Küche.</t>
         </is>
       </c>
       <c r="AF60" t="inlineStr">
         <is>
-          <t>Plants &amp; Cakes Store is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Vegan, plant-based café and restaurant in Frankfurt am Main offering bowls, cakes, breakfast dishes, snacks, and creative plant-based cuisine.</t>
         </is>
       </c>
       <c r="AG60" t="inlineStr">
         <is>
-          <t>Plants &amp; Cakes Store es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Cafetería y restaurante vegano en Fráncfort del Meno con bowls, tartas, desayunos, snacks y cocina vegetal creativa.</t>
         </is>
       </c>
       <c r="AI60" t="b">
@@ -9974,17 +9974,17 @@
       </c>
       <c r="AE61" t="inlineStr">
         <is>
-          <t>Seidenzucker Glutenfreie Patisserie &amp; Café ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Wiesbaden mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF61" t="inlineStr">
         <is>
-          <t>Seidenzucker Glutenfreie Patisserie &amp; Café is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Wiesbaden offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG61" t="inlineStr">
         <is>
-          <t>Seidenzucker Glutenfreie Patisserie &amp; Café es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Wiesbaden con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI61" t="b">
@@ -10203,17 +10203,17 @@
       </c>
       <c r="AE62" t="inlineStr">
         <is>
-          <t>NOglla glutenfreie Genussmanufaktur ist als vollständig glutenfreier Betrieb für CeliacSafe geeignet; Aufnahme konservativ auf Basis offizieller bzw. starker Spezialquellen.</t>
+          <t>Bäckerei/Patisserie in Lorch mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AF62" t="inlineStr">
         <is>
-          <t>NOglla glutenfreie Genussmanufaktur is suitable for CeliacSafe as a dedicated gluten-free venue; included conservatively based on official and/or strong specialist sources.</t>
+          <t>Bakery and patisserie in Lorch offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
         </is>
       </c>
       <c r="AG62" t="inlineStr">
         <is>
-          <t>NOglla glutenfreie Genussmanufaktur es apto para CeliacSafe como local completamente sin gluten; incluido de forma conservadora con fuentes oficiales o especializadas.</t>
+          <t>Panadería y pastelería en Lorch con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
         </is>
       </c>
       <c r="AI62" t="b">

</xml_diff>